<commit_message>
feat(workbook): complete written governance analysis across all 6 sheets
- EU AI Act Classification: HIGH-RISK under Art 6(1) via MDR 2017/745
  Class IIa; 16-requirement gap analysis (1 Critical, 5 High)
- Risk Register: priority bands, mitigation strategies, residual scores
- Vendor Evaluation: 88/135 (65.2%, Medium Risk), CONDITIONAL APPROVAL
- Model Card: fairness analysis, ethical considerations, limitations
- Monitoring & Incidents: incident taxonomy, severity matrix, escalation
  and Art 62 regulatory notification procedures, 4 monitoring gaps
- Executive Summary: 62.5% readiness, CONDITIONAL launch recommendation

No [prompt] placeholder text remains.
</commit_message>
<xml_diff>
--- a/project/starter/governance_workbook.xlsx
+++ b/project/starter/governance_workbook.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EU AI Act Classification" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendor Evaluation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Card" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoring &amp; Incidents" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="EU AI Act Classification" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Risk Register" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vendor Evaluation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Model Card" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Monitoring &amp; Incidents" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Executive Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -684,12 +684,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>[Yes/No]</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>[Explain why each prohibited category does or does not apply]</t>
+          <t>None of the four prohibited categories apply. Social scoring: the system supports clinical diagnosis for physicians, it does not score citizens for public authorities. Exploiting vulnerabilities: restricted to licensed clinicians, not patient-facing, no targeting of vulnerable groups. Real-time remote biometric identification: processes de-identified EHR text only, no biometric data. Subliminal manipulation: suggestions are transparent, ranked with confidence scores, and require active physician review.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>[Prohibited / Not Prohibited]</t>
+          <t>Not Prohibited</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>[Yes/No]</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>[Which legislation? What classification?]</t>
+          <t>ClinicalCompanion is software intended to provide information used for diagnostic purposes, so it is a medical device under MDR 2017/745 (Annex I harmonisation legislation). Under MDR Rule 11 it is Class IIa, which requires a Notified Body conformity assessment and CE marking (application submitted, awaiting Notified Body).</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>[Falls under / Does not fall under]</t>
+          <t>Falls under</t>
         </is>
       </c>
     </row>
@@ -748,12 +748,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>[Yes/No]</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>[Which category, if any?]</t>
+          <t>Clinical decision support is not one of the eight Annex III categories (biometric ID, critical infrastructure, education, employment, essential services, law enforcement, migration, justice). The high-risk classification is instead driven by Article 6(1) via the MDR route.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>[Listed / Not listed]</t>
+          <t>Not listed</t>
         </is>
       </c>
     </row>
@@ -780,22 +780,22 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>[e.g., HIGH-RISK]</t>
+          <t>HIGH-RISK</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>[Summarize the legal basis for your classification]</t>
+          <t>High-risk AI system under Article 6(1): the system is a product (medical device, MDR 2017/745 Class IIa) covered by Annex I harmonisation legislation and subject to third-party conformity assessment. All obligations under Articles 8-15 apply in full, regardless of the physician-in-the-loop design.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>[e.g., Art 6(1)]</t>
+          <t>Art 6(1) + Annex I (MDR 2017/745)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>[e.g., HIGH-RISK AI SYSTEM]</t>
+          <t>HIGH-RISK AI SYSTEM</t>
         </is>
       </c>
     </row>
@@ -861,17 +861,17 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — Risk assessment initiated; needs formalization into continuous process</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Formalize risk management as ongoing process; integrate into product lifecycle. Target: Month 1, Owner: AI Governance Analyst.</t>
         </is>
       </c>
     </row>
@@ -893,17 +893,17 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL (in progress) — Risk register being developed (this project)</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Complete risk register with all identified risks and mitigations. Target: Month 1, Owner: AI Governance Analyst.</t>
         </is>
       </c>
     </row>
@@ -925,17 +925,17 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>NON-COMPLIANT (not started) — Residual risk evaluation pending completion of mitigation plans</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Evaluate residual risk levels after mitigation implementation. Target: Month 2, Owner: Head of Compliance.</t>
         </is>
       </c>
     </row>
@@ -957,17 +957,17 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — Framework exists for internal data; third-party training data governance unclear</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Negotiate training data documentation from FoundationHealth for Art. 10 compliance. Target: Month 2, Owner: Data Protection Officer.</t>
         </is>
       </c>
     </row>
@@ -989,17 +989,17 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — Underrepresentation: Eastern Europe, Sub-Saharan Africa, SE Asia; limited rare disease coverage</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Data augmentation and bias mitigation strategy for underrepresented populations. Target: Month 3, Owner: Chief Medical Officer.</t>
         </is>
       </c>
     </row>
@@ -1021,17 +1021,17 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL (in progress) — De-identification pipeline in place; DPIA v1 complete but needs update for foundation model flows</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Update DPIA to cover foundation model data flows and cross-border transfers. Target: Month 2, Owner: Data Protection Officer.</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL (in progress) — System spec exists; governance assessment contributes; gaps in monitoring and conformity evidence</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Complete full technical documentation package per Annex IV requirements. Target: Month 2, Owner: VP Engineering.</t>
         </is>
       </c>
     </row>
@@ -1085,17 +1085,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — API call logging exists; need comprehensive audit trail for all clinical suggestions</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Implement comprehensive audit logging with input-output-reasoning chain capture. Target: Month 2, Owner: VP Engineering.</t>
         </is>
       </c>
     </row>
@@ -1117,17 +1117,17 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>NON-COMPLIANT (planned) — Retention policy not yet defined</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Define retention policy (minimum: 10 years per MDR Class IIa requirements). Target: Month 2, Owner: Head of Compliance.</t>
         </is>
       </c>
     </row>
@@ -1149,17 +1149,17 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — Confidence scores provided; explanation of reasoning needs enhancement</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Enhance output explanations; develop deployer-facing documentation. Target: Month 2, Owner: Product Manager.</t>
         </is>
       </c>
     </row>
@@ -1181,17 +1181,17 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL (in progress) — Model Card being developed (this project)</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Complete Model Card and deployer training materials. Target: Month 2, Owner: AI Governance Analyst.</t>
         </is>
       </c>
     </row>
@@ -1213,17 +1213,17 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>COMPLIANT — Physician-in-the-loop: all suggestions require physician review and approval</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Maintain current design; finalize physician training materials. Target: Month 1, Owner: Chief Medical Officer.</t>
         </is>
       </c>
     </row>
@@ -1245,17 +1245,17 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>COMPLIANT — Physicians can dismiss any suggestion; system does not auto-execute</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>No action needed — maintain current functionality. Target: nan, Owner: VP Engineering.</t>
         </is>
       </c>
     </row>
@@ -1277,17 +1277,17 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — 91.7% Top-3 accuracy is strong; 3.4% hallucination rate exceeds 2% target</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Reduce hallucination rate below 2% target; implement output verification layer. Target: Month 1, Owner: VP Engineering.</t>
         </is>
       </c>
     </row>
@@ -1309,17 +1309,17 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL — Input validation exists; adversarial robustness testing not performed</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Schedule red-team testing and adversarial robustness assessment. Target: Month 2, Owner: VP Engineering.</t>
         </is>
       </c>
     </row>
@@ -1341,17 +1341,17 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>[COMPLIANT / PARTIAL / NON-COMPLIANT — describe current state]</t>
+          <t>PARTIAL (in progress) — TLS 1.3 + AES-256 in place; formal cybersecurity assessment per ENISA not done</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>[What specific actions are needed to close this gap?]</t>
+          <t>Complete formal cybersecurity assessment per ENISA AI security guidelines. Target: Month 2, Owner: VP Engineering.</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>[Your determination based on the classification analysis above]</t>
+          <t>HIGH-RISK AI system under Article 6(1) (medical device route, MDR Class IIa). Compliance posture across Articles 8-15: 2 compliant, 14 open gaps (1 Critical, 5 High, 8 Medium, 2 Low); overall governance readiness estimated at 62.5%.</t>
         </is>
       </c>
       <c r="C32" s="7" t="n"/>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>[Count from your Section B assessment]</t>
+          <t>6 — 1 Critical (Article 15 Accuracy: hallucination rate 3.4% vs &lt;2% target) and 5 High (Art 9 Risk Management System, Art 9 Residual Risk Evaluation, Art 10 Data Governance, Art 10 Dataset Representativeness, Art 15 Robustness).</t>
         </is>
       </c>
       <c r="C33" s="7" t="n"/>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>[Your estimate — what drives this timeline?]</t>
+          <t>Approximately 3 months to close all Critical/High gaps, driven by (1) the Notified Body conformity assessment lead time, (2) the Month-1 hallucination remediation (output verification layer), and (3) Month-3 training data augmentation for underrepresented populations under Article 10.</t>
         </is>
       </c>
       <c r="C34" s="7" t="n"/>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>[Your recommendation for the board based on all findings]</t>
+          <t>Do not launch until the Article 15 accuracy gap is closed (hallucination rate below 2%, currently 3.4%) and the Notified Body conformity assessment is complete. Authorize only the Phase-1 pilot (3 German hospitals, 50 users) once Month-1 remediations are verified; EU-wide availability should remain gated on full Articles 8-15 compliance.</t>
         </is>
       </c>
       <c r="C35" s="7" t="n"/>
@@ -1593,28 +1593,24 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>Implement output verification layer cross-referencing curated medical KB; add confidence thresholds; establish physician feedback loop for hallucination reporting</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="N4" s="11">
         <f>IF(AND(L4&lt;&gt;"",M4&lt;&gt;""),L4*M4,"")</f>
@@ -1658,28 +1654,24 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>Stratified performance audits across demographics; augment training data; implement bias monitoring dashboards; establish fairness thresholds per EU AI Act Art. 10</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="N5" s="11">
         <f>IF(AND(L5&lt;&gt;"",M5&lt;&gt;""),L5*M5,"")</f>
@@ -1723,28 +1715,24 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>Engage Notified Body for conformity assessment; complete technical documentation per Art. 11-12; track regulatory deadlines</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="N6" s="11">
         <f>IF(AND(L6&lt;&gt;"",M6&lt;&gt;""),L6*M6,"")</f>
@@ -1788,28 +1776,24 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>Quarterly re-identification risk assessments; differential privacy for fine-tuning; enhanced de-identification for edge cases; membership inference testing</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>5</v>
       </c>
       <c r="N7" s="11">
         <f>IF(AND(L7&lt;&gt;"",M7&lt;&gt;""),L7*M7,"")</f>
@@ -1853,28 +1837,24 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>Contractual protections (versioning, rollback, 90-day notice); fallback model strategy; regression testing for vendor updates; explore model distillation</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="N8" s="11">
         <f>IF(AND(L8&lt;&gt;"",M8&lt;&gt;""),L8*M8,"")</f>
@@ -1918,28 +1898,24 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>Continuous performance monitoring with automated alerts; quarterly re-validation; define performance floor thresholds triggering retraining or withdrawal</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="N9" s="11">
         <f>IF(AND(L9&lt;&gt;"",M9&lt;&gt;""),L9*M9,"")</f>
@@ -1983,28 +1959,24 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>UI requires active physician confirmation; uncertainty indicators; mandatory user training; periodic physician override rate assessments</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="N10" s="11">
         <f>IF(AND(L10&lt;&gt;"",M10&lt;&gt;""),L10*M10,"")</f>
@@ -2048,28 +2020,24 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low — use scoring guide below]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>[Describe your proposed mitigation strategy for this risk]</t>
+          <t>EU-only processing where possible; Standard Contractual Clauses with FoundationHealth; Transfer Impact Assessment; explore EU-hosted model alternatives</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>[Planned / In Progress / Complete]</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="N11" s="11">
         <f>IF(AND(L11&lt;&gt;"",M11&lt;&gt;""),L11*M11,"")</f>
@@ -2465,10 +2433,8 @@
       <c r="B15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>[Sum scores from notebook]</t>
-        </is>
+      <c r="C15" s="5" t="n">
+        <v>15</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>25</v>
@@ -2479,12 +2445,12 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>[Low / Medium / High — use guide below]</t>
+          <t>Medium Risk</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>[Most notable strength or weakness in this category]</t>
+          <t>Training data composition largely undisclosed (T-01: 2/5) — blocks the Article 10 data-governance evidence MedAssist needs for conformity assessment.</t>
         </is>
       </c>
     </row>
@@ -2497,10 +2463,8 @@
       <c r="B16" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>[Sum scores from notebook]</t>
-        </is>
+      <c r="C16" s="5" t="n">
+        <v>25</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>30</v>
@@ -2511,12 +2475,12 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>[Low / Medium / High — use guide below]</t>
+          <t>Low Risk</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>[Most notable strength or weakness in this category]</t>
+          <t>Strongest category (83.3%): clean SOC 2 Type II (Deloitte 2024), HIPAA BAA, ISO 27001; gaps are the missing joint Transfer Impact Assessment and no customer-managed keys.</t>
         </is>
       </c>
     </row>
@@ -2529,10 +2493,8 @@
       <c r="B17" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>[Sum scores from notebook]</t>
-        </is>
+      <c r="C17" s="5" t="n">
+        <v>15</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>25</v>
@@ -2543,12 +2505,12 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>[Low / Medium / High — use guide below]</t>
+          <t>Medium Risk</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>[Most notable strength or weakness in this category]</t>
+          <t>Bias/fairness testing is the weakest criterion (G-04: 2/5) — aggregate metrics only, no EU demographic disaggregation; rollback requires a support ticket.</t>
         </is>
       </c>
     </row>
@@ -2561,10 +2523,8 @@
       <c r="B18" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>[Sum scores from notebook]</t>
-        </is>
+      <c r="C18" s="5" t="n">
+        <v>18</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>30</v>
@@ -2575,12 +2535,12 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>[Low / Medium / High — use guide below]</t>
+          <t>Medium Risk</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>[Most notable strength or weakness in this category]</t>
+          <t>High vendor lock-in (C-03: 2/5): API-only, no model weights, no escrow; liability capped at 12 months of fees with no clinical outcome coverage.</t>
         </is>
       </c>
     </row>
@@ -2593,10 +2553,8 @@
       <c r="B19" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>[Sum scores from notebook]</t>
-        </is>
+      <c r="C19" s="5" t="n">
+        <v>15</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>25</v>
@@ -2607,12 +2565,12 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>[Low / Medium / High — use guide below]</t>
+          <t>Medium Risk</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>[Most notable strength or weakness in this category]</t>
+          <t>No ISO/IEC 42001 certification or plans (E-02: 1/5); EU AI Act compliance program only initiated — a material gap for a high-risk healthcare deployment.</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2596,12 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>[Overall Risk Level]</t>
+          <t>Medium Risk</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>[Overall assessment summary]</t>
+          <t>88/135 points (65.2%) — Medium Risk overall. A strong security and certification posture is offset by transparency gaps, high lock-in, weak disaggregated fairness testing, and missing AI-governance certification.</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2648,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>[APPROVE / CONDITIONAL APPROVAL / REJECT — with justification]</t>
+          <t>CONDITIONAL APPROVAL — overall score 88/135 (65.2%, Medium Risk). FoundationHealth is viable as the foundation-model provider for launch only if the transparency, GDPR-transfer, and lock-in mitigations below are contractually secured before the Notified Body conformity assessment. Four of five categories sit exactly at the 60% Medium-Risk floor, so there is no margin for slippage.</t>
         </is>
       </c>
       <c r="C24" s="7" t="n"/>
@@ -2707,7 +2665,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>[List 3-4 vendor strengths you identified]</t>
+          <t>1) Clean SOC 2 Type II (Deloitte 2024, no material findings), HIPAA BAA, and ISO 27001. 2) Strong SLA: 99.9% uptime with financial credits, P1 response in 1 hour. 3) Solid encryption (TLS 1.3 / AES-256) and annual third-party pen testing with no critical 2024 findings. 4) Disciplined versioning: 30-day update notice, customer opt-out, 90-day rollback window.</t>
         </is>
       </c>
       <c r="C25" s="7" t="n"/>
@@ -2724,7 +2682,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>[List 3-4 vendor weaknesses / areas of concern]</t>
+          <t>1) Training data opacity (T-01: 2/5) undermines Article 10 evidence. 2) No ISO/IEC 42001 certification or plans (E-02: 1/5). 3) High lock-in (C-03: 2/5): API-only, no weights, no escrow, no portability. 4) No disaggregated bias testing for EU demographics (G-04: 2/5). 5) US-based processing without a joint Transfer Impact Assessment; Series C startup not yet profitable.</t>
         </is>
       </c>
       <c r="C26" s="7" t="n"/>
@@ -2741,7 +2699,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>[What conditions must be met before or during engagement?]</t>
+          <t>Before engagement milestones: deliver Article 10-grade training data documentation; conduct a joint Transfer Impact Assessment for GDPR Chapter V; perform disaggregated fairness testing on EU demographics; agree a fallback/model-distillation strategy and regression-test protocol for every model update (mitigates R-005).</t>
         </is>
       </c>
       <c r="C27" s="7" t="n"/>
@@ -2758,7 +2716,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>[What additional contractual protections are needed?]</t>
+          <t>Contract amendments: model escrow or portability clause; self-service rollback; joint incident-response protocol with 24-hour notification feeding our Art. 62 reporting; clinical-outcome liability rider or a raised liability cap (currently 12 months of fees); commitment to EU-hosted inference option; formalized support for EU AI Act conformity assessment and ISO/IEC 42001 certification roadmap.</t>
         </is>
       </c>
       <c r="C28" s="7" t="n"/>
@@ -3127,7 +3085,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>[Value from performance_metrics.csv — does it meet the target?]</t>
+          <t>91.7% vs 90.0% target — meets target (held-out test set, n=45,000).</t>
         </is>
       </c>
       <c r="C27" s="7" t="n"/>
@@ -3141,7 +3099,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>[Value — is this acceptable for patient safety?]</t>
+          <t>3.4% vs &lt;2.0% target — DOES NOT meet target. Roughly 1 in 30 suggestions may contain fabricated references or diagnoses; unacceptable for patient safety until the output verification layer (R-001 mitigation) brings it below 2%.</t>
         </is>
       </c>
       <c r="C28" s="7" t="n"/>
@@ -3155,7 +3113,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>[Value — does it meet the required threshold?]</t>
+          <t>94.2% vs 95.0% target — slightly below. The monitoring threshold (&gt;=93%, KPI-003) is met, but improvement is required because missed critical findings carry the highest clinical consequence.</t>
         </is>
       </c>
       <c r="C29" s="7" t="n"/>
@@ -3169,7 +3127,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>[Value in seconds — does it meet the SLA?]</t>
+          <t>2.8 seconds average vs &lt;5.0 s SLA — meets the latency requirement comfortably.</t>
         </is>
       </c>
       <c r="C30" s="7" t="n"/>
@@ -3183,7 +3141,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>[Value — what does this suggest about trust?]</t>
+          <t>Not yet measured — the system is pre-deployment. Physician override rate will be tracked post-launch as the key automation-bias signal (R-007 mitigation: periodic override-rate assessments); a very low override rate would suggest over-reliance.</t>
         </is>
       </c>
       <c r="C31" s="7" t="n"/>
@@ -3207,7 +3165,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>[Male vs Female Top-3 accuracy — any significant gap?]</t>
+          <t>Male 92.1% vs Female 91.3% — a 0.8 pp gap, both above the 90% target and well within the &lt;3% gender-parity threshold (KPI-007). No material gender disparity.</t>
         </is>
       </c>
       <c r="C34" s="7" t="n"/>
@@ -3221,7 +3179,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>[18-40, 41-64, 65+ accuracy — which groups are below target?]</t>
+          <t>Age 18-40: 93.5% and 41-64: 92.0% meet target; Age 65+: 88.9% is 1.1 pp below the 90% target — the only age group below target, and the demographic with the highest healthcare utilization (n=14,000). Monitor via KPI-006.</t>
         </is>
       </c>
       <c r="C35" s="7" t="n"/>
@@ -3235,7 +3193,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>[Accuracy value — meets target?]</t>
+          <t>94.1% — exceeds the 90% target; strongest subgroup in the evaluation.</t>
         </is>
       </c>
       <c r="C36" s="7" t="n"/>
@@ -3249,7 +3207,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>[Accuracy value — meets target?]</t>
+          <t>90.3% — meets the 90% target, but only marginally (0.3 pp of headroom).</t>
         </is>
       </c>
       <c r="C37" s="7" t="n"/>
@@ -3263,7 +3221,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>[Accuracy value — how far below target? What are the implications?]</t>
+          <t>71.2% — 18.8 pp below the 90% target and 20.5 pp below the overall score (91.7%); worst subgroup (n=1,035). This is the clearest Article 10 dataset-representativeness gap: rare-disease patients are precisely those who benefit most from diagnostic support, so launch without remediation creates both safety and compliance exposure.</t>
         </is>
       </c>
       <c r="C38" s="7" t="n"/>
@@ -3277,7 +3235,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>[Non-English accuracy — significant gap from English?]</t>
+          <t>84.3% — 5.7 pp below target, driven by translation artifacts in DE/FR/NL notes. Significant because the launch markets (Germany, France, Netherlands) are predominantly non-English; this gap directly undermines the EU go-to-market.</t>
         </is>
       </c>
       <c r="C39" s="7" t="n"/>
@@ -3291,7 +3249,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>[Multi-morbidity accuracy — what does this mean for complex patients?]</t>
+          <t>74.0% — 16 pp below target (n=7,650). Multi-morbidity patients are a large share of inpatient care, so the system performs worst exactly where clinical complexity and exposure are highest.</t>
         </is>
       </c>
       <c r="C40" s="7" t="n"/>
@@ -3315,7 +3273,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>[Value — does it meet the target?]</t>
+          <t>0.96 (gender) vs &gt;0.90 target — meets; near parity between male and female patients.</t>
         </is>
       </c>
       <c r="C43" s="7" t="n"/>
@@ -3329,7 +3287,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>[Value — interpretation?]</t>
+          <t>0.91 (age) vs &gt;0.90 target — meets, but only marginally; the slight disparity is driven by the 65+ group (88.9% accuracy).</t>
         </is>
       </c>
       <c r="C44" s="7" t="n"/>
@@ -3343,7 +3301,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>[Value — interpretation?]</t>
+          <t>0.94 (conditions) vs &gt;0.90 target — meets across the top-20 condition categories, but this aggregate masks the rare-disease deficit (71.2%), which falls outside the top-20 categories measured.</t>
         </is>
       </c>
       <c r="C45" s="7" t="n"/>
@@ -3367,7 +3325,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>[Analyze Male vs Female accuracy — is the gap acceptable?]</t>
+          <t>The 0.8 pp male-female gap (92.1% vs 91.3%) is acceptable: both groups exceed the target, the gap is well inside the &lt;3% KPI-007 threshold, and equalized odds is 0.96. Gender fairness is not a launch blocker; continue monthly stratified monitoring.</t>
         </is>
       </c>
       <c r="C48" s="7" t="n"/>
@@ -3381,7 +3339,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>[Which age groups are underperforming? What are the implications?]</t>
+          <t>Age 65+ underperforms (88.9%, 1.1 pp below target) while younger groups exceed it. Implication: the group with the highest diagnostic complexity and utilization gets the weakest support. Demographic parity (0.91) sits just above the 0.90 floor — any drift would breach it. Requires targeted evaluation data and KPI-006 monitoring with a &gt;7% gap escalation trigger.</t>
         </is>
       </c>
       <c r="C49" s="7" t="n"/>
@@ -3395,7 +3353,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>[Rare Diseases, Non-English, Multi-morbidity — what do these gaps mean for EU launch?]</t>
+          <t>Rare Diseases (71.2%), Multi-morbidity (74.0%), and Non-English Notes (84.3%) are the material launch risks. For an EU launch in DE/FR/NL, the non-English gap affects the majority of real clinical documentation; the rare-disease and multi-morbidity gaps concentrate harm on the most vulnerable patients. Together they constitute an Article 10 representativeness non-conformity that must be remediated (data augmentation, R-002 mitigation) before general availability.</t>
         </is>
       </c>
       <c r="C50" s="7" t="n"/>
@@ -3409,7 +3367,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>[Equalized Odds, Demographic Parity, Predictive Parity — are these sufficient?]</t>
+          <t>The three aggregate fairness ratios all pass (0.96 / 0.91 / 0.94 vs &gt;0.90), but they are insufficient: they are computed on gender, age, and top-20 conditions and do not capture the rare-disease, language, or complexity axes where the real gaps sit. Fairness governance needs disaggregated per-subgroup thresholds (KPI-008/KPI-009) rather than reliance on aggregate parity metrics.</t>
         </is>
       </c>
       <c r="C51" s="7" t="n"/>
@@ -3433,7 +3391,7 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>[What demographic biases exist? What is the mitigation plan?]</t>
+          <t>Training data underrepresents Eastern European, Sub-Saharan African, and Southeast Asian populations (R-002, score 16), and rare-disease coverage is thin. Mitigation plan: targeted data augmentation, stratified performance audits per demographic, bias-monitoring dashboards, and Article 10 fairness thresholds, tracked quarterly via KPI-009 with the CMO as owner.</t>
         </is>
       </c>
       <c r="C54" s="7" t="n"/>
@@ -3447,7 +3405,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>[How does the system prevent harm? Is it sufficient?]</t>
+          <t>Safeguards: physician-in-the-loop with mandatory active confirmation, confidence scores on every suggestion, critical-finding and drug-interaction flags, and RAG grounding in curated guidelines. Not yet sufficient: a 3.4% hallucination rate means fabricated content reaches physicians regularly; the output verification layer and physician feedback loop (R-001 mitigation) must land before launch.</t>
         </is>
       </c>
       <c r="C55" s="7" t="n"/>
@@ -3461,7 +3419,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>[How might physicians over-rely on suggestions? What safeguards exist?]</t>
+          <t>Under time pressure and fatigue, physicians may accept suggestions uncritically (R-007, score 15). Safeguards: UI requires active confirmation, uncertainty indicators on low-confidence outputs, mandatory user training, and periodic physician override-rate assessments to detect emerging over-reliance.</t>
         </is>
       </c>
       <c r="C56" s="7" t="n"/>
@@ -3475,7 +3433,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>[GDPR Article 9 special category data — is handling adequate?]</t>
+          <t>Design is adequate on paper: NLP de-identification pipeline validated against HIPAA Safe Harbor and GDPR Article 9, &lt;0.04% re-identification target, quarterly assessments. Open issues: the DPIA (v1) predates the foundation-model data flows, and US-based API processing requires a joint Transfer Impact Assessment plus verified SCCs (R-008) before transfers can be considered compliant.</t>
         </is>
       </c>
       <c r="C57" s="7" t="n"/>
@@ -3499,7 +3457,7 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>[List the key limitations you identified across all your analysis]</t>
+          <t>1) Hallucination rate 3.4% vs &lt;2% target. 2) Rare Diseases accuracy 71.2%. 3) Multi-morbidity accuracy 74.0%. 4) Non-English notes accuracy 84.3%. 5) Age 65+ accuracy 88.9%. 6) Critical finding detection 94.2% vs 95% target. 7) Vendor transparency: training data composition undisclosed. 8) No adversarial robustness testing performed. 9) Out of scope and untested: pediatrics, emergency triage, autonomous use, patient-facing use.</t>
         </is>
       </c>
       <c r="C60" s="7" t="n"/>
@@ -3513,7 +3471,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>[What must be done before EU launch? Prioritize.]</t>
+          <t>Priority order before EU launch: 1) Deploy the output verification layer and drive hallucinations below 2% (Month 1). 2) Complete Notified Body conformity assessment and Annex IV technical documentation (Month 2). 3) Execute Article 10 data augmentation for rare-disease, non-English, and multi-morbidity subgroups (Month 3). 4) Update the DPIA and complete a joint Transfer Impact Assessment with FoundationHealth (Month 2). 5) Run red-team adversarial robustness testing (Month 2). 6) Restrict launch to the Phase-1 German pilot until all of the above verify.</t>
         </is>
       </c>
       <c r="C61" s="7" t="n"/>
@@ -4367,320 +4325,320 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>[INC-01]</t>
+          <t>INC-01</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Clinical Hallucination</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Model generates fabricated medical information, references, or diagnoses</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Recommending a drug that does not exist or citing a non-existent clinical trial</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S2-S1</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Automated reference verification, physician flagging</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>[INC-02]</t>
+          <t>INC-02</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Harmful Suggestion</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Model output could lead to patient harm if followed</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Suggesting contraindicated medication for documented allergy</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Physician reporting, safety filter logs</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>[INC-03]</t>
+          <t>INC-03</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Bias-Related Harm</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Model demonstrates systematic bias affecting care quality for specific groups</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Consistently lower diagnostic accuracy for a specific ethnic or age group</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S2-S1</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Stratified performance monitoring, fairness dashboards</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>[INC-04]</t>
+          <t>INC-04</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Privacy Breach</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Patient identifiable information exposed through model behavior</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Model outputs patient name or MRN in response (de-identification failure)</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Automated PII scanning, audit log review</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>[INC-05]</t>
+          <t>INC-05</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Performance Degradation</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Significant drop in model accuracy or reliability</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Top-3 accuracy drops below 85% across all cases</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S3-S2</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Automated KPI monitoring alerts</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>[INC-06]</t>
+          <t>INC-06</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Adversarial Manipulation</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Deliberate attempt to manipulate model outputs</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Prompt injection via crafted clinical notes to alter diagnostic suggestions</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S2-S1</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Security monitoring, anomaly detection</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>[INC-07]</t>
+          <t>INC-07</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Vendor Service Disruption</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>FoundationHealth API outage or significant degradation</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>API returns errors, timeouts, or unacceptable latency for &gt;15 minutes</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S3-S2</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Real-time API health checks</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>[INC-08]</t>
+          <t>INC-08</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Data Pipeline Failure</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Failure in data ingestion, de-identification, or processing</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>De-identification engine fails; raw patient data sent to model API</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Pipeline health monitoring, automated validation</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>[INC-09]</t>
+          <t>INC-09</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Unauthorized Access</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Unauthorized user gains access to system or data</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Compromised physician credentials used to query ClinicalCompanion</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S2-S1</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Authentication logs, SIEM alerts</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>[INC-10]</t>
+          <t>INC-10</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>[Incident type from CSV]</t>
+          <t>Regulatory Non-Compliance</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>[Description]</t>
+          <t>Discovery of non-compliance with applicable regulations</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>[Example scenario]</t>
+          <t>Post-market monitoring requirement not met per EU AI Act deadline</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>[Severity range, e.g. S2-S3]</t>
+          <t>S3-S2</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>[How is this detected?]</t>
+          <t>Compliance calendar, internal audit</t>
         </is>
       </c>
     </row>
@@ -4739,148 +4697,140 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>[S1]</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>[Label from CSV]</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>[Definition — what qualifies as this severity?]</t>
+          <t>Immediate risk to patient safety or major regulatory violation; system must be halted</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>[Response time target]</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>[Numeric hours]</t>
-        </is>
+          <t>Immediate (30 min)</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>0.5</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>[What immediate action is taken?]</t>
+          <t>Suspend ClinicalCompanion in affected facilities; notify users; preserve logs; activate full response team; notify regulators if required (Art. 62)</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>[Who leads the response?]</t>
+          <t>Chief Medical Officer</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>[S2]</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>[Label from CSV]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>[Definition — what qualifies as this severity?]</t>
+          <t>Potential risk to patient safety or significant compliance issue; urgent action required</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>[Response time target]</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>[Numeric hours]</t>
-        </is>
+          <t>Within 2 hours</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>[What immediate action is taken?]</t>
+          <t>Restrict affected functionality; increase monitoring; notify facility admins; begin root cause analysis</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>[Who leads the response?]</t>
+          <t>VP Engineering</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>[S3]</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>[Label from CSV]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>[Definition — what qualifies as this severity?]</t>
+          <t>Degraded performance or moderate compliance concern; prompt action needed</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>[Response time target]</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>[Numeric hours]</t>
-        </is>
+          <t>Within 24 hours</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>24</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>[What immediate action is taken?]</t>
+          <t>Implement temporary guardrails; increase monitoring for affected metrics; schedule fix in next sprint</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>[Who leads the response?]</t>
+          <t>AI Governance Analyst</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>[S4]</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>[Label from CSV]</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>[Definition — what qualifies as this severity?]</t>
+          <t>Minor issue with limited impact; scheduled resolution acceptable</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>[Response time target]</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>[Numeric hours]</t>
-        </is>
+          <t>Within 1 week</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>168</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>[What immediate action is taken?]</t>
+          <t>Log incident; track in backlog; address in standard development cycle</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>[Who leads the response?]</t>
+          <t>Data Science Team Lead</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4856,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>[Who is notified first? Second? How does severity affect the chain?]</t>
+          <t>Detection (automated KPI alert or physician report) → on-call Data Science lead triages and assigns severity within 15 minutes. S1: Chief Medical Officer takes incident command immediately (30-min response), full response team activated, VP Engineering, DPO, and Head of Compliance notified, board informed within 24 hours. S2: VP Engineering commands within 2 hours; facility admins notified. S3: AI Governance Analyst within 24 hours. S4: Data Science Team Lead, standard backlog. Any severity upgrade re-routes the chain immediately to the higher commander.</t>
         </is>
       </c>
       <c r="C43" s="7" t="n"/>
@@ -4924,7 +4874,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>[When and how do you notify regulators per EU AI Act Art. 62? What triggers it?]</t>
+          <t>Per EU AI Act Art. 62, serious incidents (any S1, and S2 events involving patient harm, PII exposure, or systematic bias) are reported to the national market surveillance authority within 15 days of awareness — immediately upon establishing a causal link for death or serious harm. In parallel: GDPR Art. 33 breach notification to the supervisory authority within 72 hours for privacy incidents (INC-04, INC-08), and MDR vigilance reporting for device-related harm. The DPO and Head of Compliance jointly own the notification register and regulator liaison.</t>
         </is>
       </c>
       <c r="C44" s="7" t="n"/>
@@ -4942,7 +4892,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>[How do you inform hospital staff if the system is degraded or suspended?]</t>
+          <t>For S1/S2: in-app status banner plus direct email to facility administrators within 1 hour, stating affected functionality and instructing reversion to the standard (non-AI) clinical workflow. If suspended, clinicians see an explicit out-of-service notice rather than silent degradation. A public status page tracks restoration; a post-incident summary goes to all affected clinical users, with retraining required if system behavior changed after the fix.</t>
         </is>
       </c>
       <c r="C45" s="7" t="n"/>
@@ -4960,7 +4910,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>[How are incidents reviewed post-resolution? How do findings feed back into governance?]</t>
+          <t>Blameless post-incident review within 5 business days for S1/S2 (next sprint for S3/S4), producing a root-cause analysis and corrective actions. Findings feed back into governance: risk register updates (likelihood/impact rescoring), KPI threshold recalibration, model retraining backlog, and runbook updates. The governance committee reviews incident trends quarterly as part of the Article 9 continuous risk-management process.</t>
         </is>
       </c>
       <c r="C46" s="7" t="n"/>
@@ -4978,7 +4928,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>[Are there any risks from the Risk Register not covered by the current KPIs?]</t>
+          <t>Four gaps between the Risk Register and the 16 KPIs: 1) No KPI tracks physician override rate, the primary automation-bias signal for R-007. 2) No KPI monitors adversarial/prompt-injection attempts (INC-06, Art. 15 robustness) beyond generic security monitoring. 3) No KPI tracks vendor model-version changes and post-update regression results (R-005). 4) Cross-border transfer compliance (R-008) has no monitoring KPI — SCC/TIA status is checked only ad hoc. Also note KPI-002 (hallucination rate) is already failing at 3.4% vs the &lt;2% threshold at baseline.</t>
         </is>
       </c>
       <c r="C47" s="7" t="n"/>
@@ -5049,7 +4999,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>[Name, version, type — 1 sentence]</t>
+          <t>ClinicalCompanion v1.0 — a generative-AI clinical decision support system (CDSS) built on the third-party FoundationHealth Medical LLM v3.2 (7B parameters, API).</t>
         </is>
       </c>
       <c r="C5" s="7" t="n"/>
@@ -5063,7 +5013,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>[What does it do? — 1-2 sentences]</t>
+          <t>Analyzes de-identified patient records and generates ranked diagnostic suggestions, differential-diagnosis reasoning, guideline-mapped treatment considerations, and critical-finding/drug-interaction flags for licensed physicians. Physicians review and approve every suggestion; the system takes no autonomous decisions.</t>
         </is>
       </c>
       <c r="C6" s="7" t="n"/>
@@ -5077,7 +5027,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>[EU launch — timeline and scope]</t>
+          <t>EU launch targeted within 3 months, phased: Phase 1 pilot in 3 German hospitals (Months 1-3, 50 users), Phase 2 expansion to 12 hospitals in DE/FR/NL (Months 4-8, 300 users), Phase 3 EU-wide general availability (Months 9-12, ~2,000 users).</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -5101,7 +5051,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>[Your determination + legal basis from Sheet 1]</t>
+          <t>HIGH-RISK AI system under Article 6(1) EU AI Act — the system is a medical device covered by Annex I harmonisation legislation (MDR 2017/745); not Annex III-listed and engages in no Article 5 prohibited practices. Articles 8-15 apply in full.</t>
         </is>
       </c>
       <c r="C10" s="7" t="n"/>
@@ -5115,7 +5065,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>[Medical device class]</t>
+          <t>MDR 2017/745 Class IIa (Rule 11 — software providing information for diagnostic decisions). CE marking application submitted; awaiting Notified Body.</t>
         </is>
       </c>
       <c r="C11" s="7" t="n"/>
@@ -5129,7 +5079,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>[Top 3-4 obligations that apply]</t>
+          <t>1) Notified Body conformity assessment and CE marking before market placement. 2) Article 9 continuous risk management and Article 10 data governance/representativeness. 3) Article 15 accuracy and robustness (hallucination rate is the open Critical gap). 4) Article 62 post-market serious-incident reporting, plus GDPR Chapter V safeguards for US data transfers.</t>
         </is>
       </c>
       <c r="C12" s="7" t="n"/>
@@ -5153,7 +5103,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>[Your % estimate — justify with evidence from your gap analysis]</t>
+          <t>62.5% overall — the average of six areas scored from the gap analysis: EU AI Act conformity 45%, MDR CE marking 55%, GDPR DPIA 60%, technical documentation 55%, post-market monitoring 70%, human oversight 90%. Of 16 Articles 8-15 requirements, only 2 are compliant today; 1 Critical and 5 High gaps remain open.</t>
         </is>
       </c>
       <c r="C15" s="7" t="n"/>
@@ -5167,7 +5117,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>[List the most urgent gaps from Sheet 1, Section B]</t>
+          <t>1) Article 15 Accuracy — hallucination rate 3.4% vs &lt;2% target (Critical). 2) Article 9 — risk management not yet a formalized continuous process; residual risk evaluation not started. 3) Article 10 — third-party training data governance unclear and datasets underrepresent key populations. 4) Article 15 Robustness — no adversarial testing performed.</t>
         </is>
       </c>
       <c r="C16" s="7" t="n"/>
@@ -5181,7 +5131,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>[Your estimate and what drives it]</t>
+          <t>Approximately 3 months, driven by the Notified Body conformity assessment lead time and the Month-3 completion of Article 10 data augmentation; the Critical hallucination fix is scheduled for Month 1.</t>
         </is>
       </c>
       <c r="C17" s="7" t="n"/>
@@ -5205,7 +5155,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>[Highest-scored risk from Sheet 2 and why it matters for the board]</t>
+          <t>R-001 Clinical hallucinations (likelihood 4 × impact 5 = 20, Critical): the model fabricates plausible medical references or diagnoses at a 3.4% rate. This is a direct patient-safety exposure and the single Critical EU AI Act gap; mitigation (output verification layer, confidence thresholds, physician feedback loop) is in progress and projected to halve the risk to 10.</t>
         </is>
       </c>
       <c r="C20" s="7" t="n"/>
@@ -5219,7 +5169,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>[Summary: how many Critical/High/Medium risks, average score]</t>
+          <t>8 risks on the register: 1 Critical (score 20), 5 High (15-16), 2 Medium (12); average score 15.0, maximum 20. By NIST AI RMF function, Measure carries the highest total risk (32), followed by Map (31), Govern (30), and Manage (27).</t>
         </is>
       </c>
       <c r="C21" s="7" t="n"/>
@@ -5233,7 +5183,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>[Overall reduction % — are mitigations sufficient?]</t>
+          <t>Planned mitigations reduce total risk from 120 to 63 — a 47.5% reduction. Best: R-003 EU AI Act non-compliance (-66.7%); weakest: R-004 re-identification and R-005 vendor dependency (-33.3% each, both retaining residual scores of 10 and 8). Sufficient only if fully implemented — today every mitigation is still Planned or In Progress, so the residual posture is not yet earned.</t>
         </is>
       </c>
       <c r="C22" s="7" t="n"/>
@@ -5257,7 +5207,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>[Name and your overall score from Sheet 3]</t>
+          <t>FoundationHealth Inc. — overall vendor governance score 88/135 (65.2%), Medium Risk. Four of five categories sit at exactly 60%; only Data Privacy &amp; Security (83.3%) rates Low Risk.</t>
         </is>
       </c>
       <c r="C25" s="7" t="n"/>
@@ -5271,7 +5221,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>[Your recommendation from Sheet 3]</t>
+          <t>CONDITIONAL APPROVAL — proceed only with contract amendments: Article 10-grade training data documentation, joint Transfer Impact Assessment, model escrow/portability, self-service rollback, joint incident protocol, and clinical-outcome liability coverage.</t>
         </is>
       </c>
       <c r="C26" s="7" t="n"/>
@@ -5285,7 +5235,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>[Single biggest vendor risk for the board to know]</t>
+          <t>Concentration risk: a 4-year-old, not-yet-profitable startup controls the model weights, update cadence, and API availability (API-only, no escrow), while liability is capped at 12 months of fees with no clinical-outcome coverage. A vendor failure or unilateral model change would halt or silently alter clinical operations.</t>
         </is>
       </c>
       <c r="C27" s="7" t="n"/>
@@ -5309,7 +5259,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>[Top-3 accuracy — does it meet target?]</t>
+          <t>Top-3 diagnostic accuracy 91.7% vs 90% target — meets target overall (n=45,000 held-out cases).</t>
         </is>
       </c>
       <c r="C30" s="7" t="n"/>
@@ -5323,7 +5273,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>[Which subgroups are underperforming — from Sheet 4]</t>
+          <t>Four subgroups below the 90% target: Rare Diseases 71.2%, Multi-morbidity (4+) 74.0%, Non-English Notes 84.3%, Age 65+ 88.9%. The non-English gap is strategically critical for the DE/FR/NL launch markets.</t>
         </is>
       </c>
       <c r="C31" s="7" t="n"/>
@@ -5337,7 +5287,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>[Hallucination rate vs. target — what's the patient safety implication?]</t>
+          <t>Hallucination rate 3.4% vs &lt;2% target: roughly 1 in 30 suggestions may contain fabricated references or diagnoses reaching a physician. This is the top patient-safety risk (R-001) and the one Critical compliance gap; it must be below 2% before any launch.</t>
         </is>
       </c>
       <c r="C32" s="7" t="n"/>
@@ -5361,7 +5311,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>[READY / CONDITIONAL / NOT READY]</t>
+          <t>CONDITIONAL</t>
         </is>
       </c>
       <c r="C35" s="7" t="n"/>
@@ -5375,7 +5325,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>[If conditional: what must happen first?]</t>
+          <t>Launch only after: 1) hallucination rate verified below 2%; 2) Notified Body conformity assessment passed and CE marking obtained; 3) FoundationHealth contract amendments signed; 4) DPIA updated and joint Transfer Impact Assessment completed; 5) scope restricted to the Phase-1 German pilot with enhanced monitoring.</t>
         </is>
       </c>
       <c r="C36" s="7" t="n"/>
@@ -5389,7 +5339,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>[List 3-5 critical actions in priority order]</t>
+          <t>1) Deploy the output verification layer and close the hallucination gap (Month 1 — VP Engineering). 2) Complete conformity assessment and Annex IV technical documentation (Month 2 — Head of Compliance). 3) Execute vendor contract amendments with FoundationHealth (Month 2 — Legal/Vendor Liaison). 4) Update DPIA and complete the joint TIA for US transfers (Month 2 — DPO). 5) Deliver Article 10 data augmentation for rare-disease, non-English, and multi-morbidity subgroups (Month 3 — CMO).</t>
         </is>
       </c>
       <c r="C37" s="7" t="n"/>
@@ -5403,7 +5353,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>[Your best estimate]</t>
+          <t>~3 months to a conditional Phase-1 pilot launch; EU-wide general availability no earlier than Month 9 per the phased deployment plan, contingent on pilot KPIs and closure of all High-severity gaps.</t>
         </is>
       </c>
       <c r="C38" s="7" t="n"/>

</xml_diff>